<commit_message>
Simplify PET history table and add Lugano column
</commit_message>
<xml_diff>
--- a/pacjenci/ADAM WOSIK.xlsx
+++ b/pacjenci/ADAM WOSIK.xlsx
@@ -483,7 +483,11 @@
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Inne</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>Do oceny</t>
@@ -523,10 +527,14 @@
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Inne</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Brak aktywnej choroby</t>
+          <t>Do oceny</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -534,17 +542,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3 - wychwyt nie większy niż wątroba</t>
+          <t>4 - utrzymujący się wychwyt patologiczny</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Nie stwierdza się aktywnej metabolicznie choroby. Klasyfikacja Lugano: Complete Response (CR) - całkowita odpowiedź na leczenie. Deauville: 3 - wychwyt nie większy niż wątroba.</t>
+          <t>Stabilizacja choroby. Klasyfikacja Lugano: Stable Disease (SD) - stabilizacja choroby. Deauville: 4 - utrzymujący się wychwyt patologiczny.</t>
         </is>
       </c>
     </row>
@@ -614,7 +622,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Brak aktywnej choroby</t>
+          <t>Do oceny</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -622,17 +630,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3 - wychwyt nie większy niż wątroba</t>
+          <t>4 - utrzymujący się wychwyt patologiczny</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Nie stwierdza się aktywnej metabolicznie choroby. Klasyfikacja Lugano: Complete Response (CR) - całkowita odpowiedź na leczenie. Deauville: 3 - wychwyt nie większy niż wątroba.</t>
+          <t>Stabilizacja choroby. Klasyfikacja Lugano: Stable Disease (SD) - stabilizacja choroby. Deauville: 4 - utrzymujący się wychwyt patologiczny.</t>
         </is>
       </c>
     </row>

</xml_diff>